<commit_message>
Add settlement and onboarding completion webhook functionality
Add webhooks for settlement completion and onboarding completion, including HMAC-SHA256 signed payloads, to `server/services/bondaiSettlementWebhook.ts` and `server/external-onboarding.ts`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 475f8ebc-5ba0-4d5e-8a54-28dbc75b1230
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ca1faf34-539d-4331-97f7-71429b2feff2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8f4ec8c9-4e63-449d-96ac-18253f3aadd8/475f8ebc-5ba0-4d5e-8a54-28dbc75b1230/sf79kCG
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/JACE_CRM_Complete_Project_Updates.xlsx
+++ b/JACE_CRM_Complete_Project_Updates.xlsx
@@ -1360,7 +1360,7 @@
         <v>Voice Assistant Widget</v>
       </c>
       <c r="E56" t="str">
-        <v>OpenAI speech-to-text (gpt-4o-mini-transcribe) and text-to-speech (gpt-audio with 'nova' voice), microphone recording and audio playback</v>
+        <v>OpenAI speech-to-text (gpt-4o-mini-transcribe) and text-to-speech (gpt-audio with nova voice), microphone recording and audio playback</v>
       </c>
     </row>
     <row r="57">
@@ -1377,7 +1377,7 @@
         <v>Voice Assistant on All Pages</v>
       </c>
       <c r="E57" t="str">
-        <v>Floating 'Voice Help' button available on all authenticated pages via global widget</v>
+        <v>Floating Voice Help button available on all authenticated pages via global widget</v>
       </c>
     </row>
     <row r="58">
@@ -1530,7 +1530,7 @@
         <v>Settlement Submit Endpoint</v>
       </c>
       <c r="E66" t="str">
-        <v>POST /api/settlement/complete - Investor submits settlement (status: active → submitted), fires JACE_SETTLEMENT_SUBMITTED postMessage</v>
+        <v>POST /api/settlement/complete - Investor submits settlement (status: active to submitted), fires JACE_SETTLEMENT_SUBMITTED postMessage</v>
       </c>
     </row>
     <row r="67">
@@ -1581,7 +1581,7 @@
         <v>Settlement Schema</v>
       </c>
       <c r="E69" t="str">
-        <v>settlement_sessions table: id, sessionId, investorName, investorEmail, amount, currency, bondId, bondName, status, metadata, receiptPdf, confirmedBy/At, cancelledBy/At, cancellationReason, timestamps</v>
+        <v>settlement_sessions table with full audit trail columns</v>
       </c>
     </row>
     <row r="70">
@@ -1700,7 +1700,7 @@
         <v>Settlement Summary Endpoint</v>
       </c>
       <c r="E76" t="str">
-        <v>GET /api/admin/settlements/summary - Count of settlements by status (submitted, confirmed, cancelled, active)</v>
+        <v>GET /api/admin/settlements/summary - Count of settlements by status</v>
       </c>
     </row>
     <row r="77">
@@ -1785,7 +1785,7 @@
         <v>Settlement Webhook Service</v>
       </c>
       <c r="E81" t="str">
-        <v>HMAC-SHA256 signed webhook to BondAI for settlement.completed event (sessionId, investorName, amount, currency, confirmedBy, confirmedAt)</v>
+        <v>HMAC-SHA256 signed webhook to BondAI for settlement.completed event</v>
       </c>
     </row>
     <row r="82">
@@ -2181,7 +2181,7 @@
         <v>POST</v>
       </c>
       <c r="C4" t="str">
-        <v>Investor submits settlement (active → submitted)</v>
+        <v>Investor submits settlement (active to submitted)</v>
       </c>
       <c r="D4" t="str">
         <v>JWT Token</v>
@@ -2454,7 +2454,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Webhook / Event</v>
+        <v>Webhook or Event</v>
       </c>
       <c r="B1" t="str">
         <v>Direction</v>
@@ -2477,7 +2477,7 @@
         <v>settlement.completed</v>
       </c>
       <c r="B2" t="str">
-        <v>JACE → BondAI</v>
+        <v>JACE to BondAI</v>
       </c>
       <c r="C2" t="str">
         <v>Admin confirms settlement</v>
@@ -2497,7 +2497,7 @@
         <v>onboarding.completed</v>
       </c>
       <c r="B3" t="str">
-        <v>JACE → BondAI</v>
+        <v>JACE to BondAI</v>
       </c>
       <c r="C3" t="str">
         <v>Investor completes onboarding</v>
@@ -2517,7 +2517,7 @@
         <v>/api/jace/investor-kyc-update</v>
       </c>
       <c r="B4" t="str">
-        <v>JACE → BondAI (Direct API)</v>
+        <v>JACE to BondAI (Direct API)</v>
       </c>
       <c r="C4" t="str">
         <v>Onboarding completion</v>
@@ -2537,7 +2537,7 @@
         <v>x-bondai-webhook-secret header</v>
       </c>
       <c r="B5" t="str">
-        <v>BondAI → JACE (Inbound)</v>
+        <v>BondAI to JACE (Inbound)</v>
       </c>
       <c r="C5" t="str">
         <v>Settlement session creation</v>
@@ -2557,7 +2557,7 @@
         <v>JACE_SETTLEMENT_LOADED</v>
       </c>
       <c r="B6" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C6" t="str">
         <v>Settlement page loads</v>
@@ -2577,13 +2577,13 @@
         <v>JACE_SETTLEMENT_SUBMITTED</v>
       </c>
       <c r="B7" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C7" t="str">
         <v>Investor submits settlement</v>
       </c>
       <c r="D7" t="str">
-        <v>{ sessionId, status: 'submitted' }</v>
+        <v>{ sessionId, status: submitted }</v>
       </c>
       <c r="E7" t="str">
         <v>Window postMessage</v>
@@ -2597,7 +2597,7 @@
         <v>JACE_SETTLEMENT_FAILED</v>
       </c>
       <c r="B8" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C8" t="str">
         <v>Settlement processing fails</v>
@@ -2617,13 +2617,13 @@
         <v>JACE_SETTLEMENT_CANCELLED</v>
       </c>
       <c r="B9" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C9" t="str">
         <v>Investor cancels settlement</v>
       </c>
       <c r="D9" t="str">
-        <v>{ sessionId, status: 'cancelled' }</v>
+        <v>{ sessionId, status: cancelled }</v>
       </c>
       <c r="E9" t="str">
         <v>Window postMessage</v>
@@ -2637,7 +2637,7 @@
         <v>JACE_ONBOARDING_COMPLETE</v>
       </c>
       <c r="B10" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C10" t="str">
         <v>Onboarding completed</v>
@@ -2657,7 +2657,7 @@
         <v>JACE_ONBOARDING_CANCEL</v>
       </c>
       <c r="B11" t="str">
-        <v>JACE iframe → BondAI (postMessage)</v>
+        <v>JACE iframe to BondAI (postMessage)</v>
       </c>
       <c r="C11" t="str">
         <v>Onboarding cancelled</v>

</xml_diff>